<commit_message>
test(excel): M_Stockist full-test plan + all-brands m_combined fixture
Adds docs/EXCEL_IMPORT_M_STOCKIST_TEST.md — a full-coverage on-device test plan
for the M (manufacturer) Excel upload path: combined multi-brand sheet + ENTRY
export, per-brand alias writes, batch-sum, map-only rows, quantity modes, the
new-design needs-fill guard, atomicity/retry-after-failure, edges, and DB
verification queries.

Extends m_combined.xlsx to carry a column for EVERY brand on the test account
(adds the default/main "cura ceramic" brand alongside BOTTEGA/CERA TILES/ENNFACE)
plus a junk "ZZ JUNKCOL" column that must be ignored — so the test proves all
real brand names land in the DB and unknown columns are dropped.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/templates/test_fixtures/m_combined.xlsx
+++ b/docs/templates/test_fixtures/m_combined.xlsx
@@ -14,11 +14,14 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="39">
   <si>
     <t>Master Design</t>
   </si>
   <si>
+    <t>cura ceramic</t>
+  </si>
+  <si>
     <t>BOTTEGA</t>
   </si>
   <si>
@@ -28,6 +31,9 @@
     <t>ENNFACE</t>
   </si>
   <si>
+    <t>ZZ JUNKCOL</t>
+  </si>
+  <si>
     <t>Size</t>
   </si>
   <si>
@@ -58,12 +64,18 @@
     <t>CLOUD ONYX</t>
   </si>
   <si>
+    <t>Cura Cloud</t>
+  </si>
+  <si>
     <t>Bottega Cloud</t>
   </si>
   <si>
     <t>Cera Onyx</t>
   </si>
   <si>
+    <t>Junk Cloud</t>
+  </si>
+  <si>
     <t>800x1600</t>
   </si>
   <si>
@@ -101,6 +113,9 @@
   </si>
   <si>
     <t>DUNE BEIGE</t>
+  </si>
+  <si>
+    <t>Cura Dune</t>
   </si>
   <si>
     <t>Bottega Dune</t>
@@ -462,16 +477,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:O4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.7109375" customWidth="1"/>
-    <col min="2" max="10" width="12.7109375" customWidth="1"/>
-    <col min="11" max="11" width="13.7109375" customWidth="1"/>
-    <col min="12" max="13" width="12.7109375" customWidth="1"/>
+    <col min="2" max="2" width="14.7109375" customWidth="1"/>
+    <col min="3" max="12" width="12.7109375" customWidth="1"/>
+    <col min="13" max="13" width="13.7109375" customWidth="1"/>
+    <col min="14" max="15" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:15">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -511,119 +527,134 @@
       <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
     </row>
-    <row r="2" spans="1:13">
+    <row r="2" spans="1:15">
       <c r="A2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C2" t="s">
-        <v>15</v>
-      </c>
-      <c r="E2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F2">
+        <v>17</v>
+      </c>
+      <c r="D2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H2">
         <v>252</v>
       </c>
-      <c r="G2">
+      <c r="I2">
         <v>0</v>
       </c>
-      <c r="H2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
+        <v>21</v>
+      </c>
+      <c r="K2" t="s">
+        <v>22</v>
+      </c>
+      <c r="L2">
+        <v>3</v>
+      </c>
+      <c r="M2">
+        <v>35</v>
+      </c>
+      <c r="N2" t="s">
+        <v>23</v>
+      </c>
+      <c r="O2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15">
+      <c r="A3" t="s">
+        <v>25</v>
+      </c>
+      <c r="E3" t="s">
+        <v>26</v>
+      </c>
+      <c r="G3" t="s">
+        <v>27</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <v>32</v>
+      </c>
+      <c r="J3" t="s">
+        <v>28</v>
+      </c>
+      <c r="K3" t="s">
+        <v>29</v>
+      </c>
+      <c r="L3">
+        <v>4</v>
+      </c>
+      <c r="M3">
+        <v>24</v>
+      </c>
+      <c r="N3" t="s">
+        <v>30</v>
+      </c>
+      <c r="O3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15">
+      <c r="A4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C4" t="s">
+        <v>34</v>
+      </c>
+      <c r="D4" t="s">
+        <v>35</v>
+      </c>
+      <c r="E4" t="s">
+        <v>36</v>
+      </c>
+      <c r="G4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H4">
+        <v>100</v>
+      </c>
+      <c r="I4">
+        <v>50</v>
+      </c>
+      <c r="J4" t="s">
+        <v>21</v>
+      </c>
+      <c r="K4" t="s">
+        <v>38</v>
+      </c>
+      <c r="L4">
+        <v>6</v>
+      </c>
+      <c r="M4">
         <v>18</v>
       </c>
-      <c r="J2">
-        <v>3</v>
-      </c>
-      <c r="K2">
-        <v>35</v>
-      </c>
-      <c r="L2" t="s">
-        <v>19</v>
-      </c>
-      <c r="M2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" t="s">
-        <v>21</v>
-      </c>
-      <c r="D3" t="s">
-        <v>22</v>
-      </c>
-      <c r="E3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F3">
-        <v>0</v>
-      </c>
-      <c r="G3">
-        <v>32</v>
-      </c>
-      <c r="H3" t="s">
+      <c r="N4" t="s">
+        <v>30</v>
+      </c>
+      <c r="O4" t="s">
         <v>24</v>
-      </c>
-      <c r="I3" t="s">
-        <v>25</v>
-      </c>
-      <c r="J3">
-        <v>4</v>
-      </c>
-      <c r="K3">
-        <v>24</v>
-      </c>
-      <c r="L3" t="s">
-        <v>26</v>
-      </c>
-      <c r="M3" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" t="s">
-        <v>28</v>
-      </c>
-      <c r="B4" t="s">
-        <v>29</v>
-      </c>
-      <c r="C4" t="s">
-        <v>30</v>
-      </c>
-      <c r="D4" t="s">
-        <v>31</v>
-      </c>
-      <c r="E4" t="s">
-        <v>32</v>
-      </c>
-      <c r="F4">
-        <v>100</v>
-      </c>
-      <c r="G4">
-        <v>50</v>
-      </c>
-      <c r="H4" t="s">
-        <v>17</v>
-      </c>
-      <c r="I4" t="s">
-        <v>33</v>
-      </c>
-      <c r="J4">
-        <v>6</v>
-      </c>
-      <c r="K4">
-        <v>18</v>
-      </c>
-      <c r="L4" t="s">
-        <v>26</v>
-      </c>
-      <c r="M4" t="s">
-        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>